<commit_message>
E72 (2.7h): PLZ aus Ort im Import, Ortsteil-Toleranz für Formular und Import (Migration 0051)
- plz_ort_norm_passt: eine Passt-Regel auf Normalformen (gleich, Kurzform,
  Ortsteil); plz_ort_passt wird zur Hülle; Spiegel ortNormPasst/ortPasst,
  Parität in plz-check (Fixture-Fälle und Messung PLZMESSUNG_ORT)
- plz_fuer_ort: PLZ-Kandidaten je Ort mit Kreis und Land über den ARS
- Import: vor dem Akteur-Abgleich PLZ aus Ort ergänzen (eine Abfrage je
  Lauf); eindeutig → PLZ + Hinweis, sonst Befund mit Kandidaten (max. zehn
  PLZ) am Feld Sitz-PLZ und Nacharbeit; Zähler plz_aus_ort/_offen
- Nacharbeit: Ort-Änderung bei leerer PLZ stößt Auflösung neu an und räumt
  nur den eigenen Befund
- Testdatei: Blatt „Testfälle" Zeilen 18/21/39 mit neuer Erwartung
- Entscheidungslog §47 (inkl. Hinweis zur Neunummerierung 0051–0054 in
  #199–#203 und neuem Journal-when)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HLRRtDF7EeEekbWYwLJdNB
</commit_message>
<xml_diff>
--- a/docs/beispiele/import-testdatei-ap27.xlsx
+++ b/docs/beispiele/import-testdatei-ap27.xlsx
@@ -3615,7 +3615,7 @@
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>Nacharbeit; 'Meinten Sie …?' mit PLZ zu Mosbach (lokal)</t>
+          <t>PLZ aus Ort ergänzt (E72 a): Mosbach ist genau einer PLZ zugeordnet → 74821 übernommen, Hinweis 'PLZ aus Ort ergänzt', Sitz-Genauigkeit plz_gebiet; Import ok</t>
         </is>
       </c>
     </row>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="D19" s="24" t="inlineStr">
         <is>
-          <t>Nacharbeit; 'Meinten Sie …?' mit Kreis und Land; ähnlich zu Preview-Akteur 'Test: Kompostwerk Breisgau'</t>
+          <t>Nacharbeit (E72 b): Befund am Feld Sitz-PLZ nennt die Kandidaten mit Kreis und Land (Freiburg (Elbe), Landkreis Stade, Niedersachsen; Freiburg im Breisgau, Stadtkreis …, PLZ-Liste max. 10); nach Wahl der PLZ läuft der Akteur-Abgleich erneut → 'Test: Kompostwerk Breisgau' als stark-Vorschlag (E72 c)</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4035,7 @@
       </c>
       <c r="D37" s="24" t="inlineStr">
         <is>
-          <t>PLZ 68199 gehört zu Mannheim → 'Meinten Sie 68199 Mannheim?' oder Ortsteil-Toleranz (Weggabelung)</t>
+          <t>Ortsteil-Toleranz (E72 e): 'Mannheim-Neckarau' beginnt mit dem amtlichen Ort Mannheim + Trennzeichen → passt zu 68199, Ort bleibt unverändert, keine Meldung; Import ok ('Mannheimer Str.' wäre ein Befund)</t>
         </is>
       </c>
     </row>

</xml_diff>